<commit_message>
Add Phase 5 dashboard UI, fix indicator directions, and restructure Health & Safety
- Dashboard: Search, Benchmark, About panels; sub-component navigation; trend pills; rank badges; number formatting; no-data trend indicator; insights button redesign; all-same-rank suppression
- Direction audit: fix 5 indicators (Board/Employees/KMP → neutral, WaterWithdrawalByOthers/Seawater → lower_is_better); patch ranks.ts isAllSameRank for all-null neutral indicators
- Health & Safety: reorder by indicator type (TRIFR/LTIFR/Fatalities/Injuries/Rehab pairs); rename TRIFR/LTIFR/Fatalities labels with Employee/Worker prefix

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parser/review/analysis_review.xlsx
+++ b/parser/review/analysis_review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Prakhar\claude code\Tata steel BRSR benchmark\parser\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502BC688-4CD2-48D5-BB35-C2D51AB869C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36D3039C-C254-4BA9-9000-F39A441A0079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="792">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="793">
   <si>
     <t>KPI</t>
   </si>
@@ -4529,6 +4529,9 @@
   <si>
     <t>Tata Steel standalone = 2.91 TCO2e
 Add in comparability note - "The number is calculated manually using GHG protocol Scope 1 and 2 divided by crude steel production of Tata Steel standalone)</t>
+  </si>
+  <si>
+    <t>"Tata Steel FY2022-23 is flagged as consolidated in the original XBRL filing, while the standalone net worth values used in this benchmark are sourced from the annual report for comparability with other standalone peer companies." - Never mention XBRL or reference to it in AI analysis or its components.</t>
   </si>
 </sst>
 </file>
@@ -5132,7 +5135,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="336" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="345.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
@@ -5164,7 +5167,9 @@
         <v>30</v>
       </c>
       <c r="K5" s="6"/>
-      <c r="L5" s="9"/>
+      <c r="L5" s="9" t="s">
+        <v>792</v>
+      </c>
     </row>
     <row r="6" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="24" t="s">
@@ -5182,7 +5187,7 @@
       <c r="K6" s="25"/>
       <c r="L6" s="25"/>
     </row>
-    <row r="7" spans="1:12" ht="90" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="390" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
@@ -5220,7 +5225,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="90" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="360" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>43</v>
       </c>

</xml_diff>